<commit_message>
longue distance: inversion de l'ordre des questions
et mise à jour de l'année dans le libellé

fixes #514
</commit_message>
<xml_diff>
--- a/survey/references/OD_nationale_quebec_2025.xlsx
+++ b/survey/references/OD_nationale_quebec_2025.xlsx
@@ -1878,16 +1878,65 @@
     <t xml:space="preserve">Custom because it is a map around the home</t>
   </si>
   <si>
-    <t xml:space="preserve">householdLongDistanceTripsSeptemberDecember</t>
-  </si>
-  <si>
-    <t xml:space="preserve">household.longDistanceTripsSeptemberDecember</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À quelle fréquence vous ou un des membres de votre ménage avez-vous effectué des déplacements longue distance (plus de 40 km) de **septembre à décembre 2024**?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How often did you or a member of your household make long-distance trips (more than 40 km) between **September and December 2024**?</t>
+    <t xml:space="preserve">householdLongDistanceTripsMayAugust</t>
+  </si>
+  <si>
+    <t xml:space="preserve">household.longDistanceTripsMayAugust</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À quelle fréquence vous ou un des membres de votre ménage avez-vous effectué des déplacements longue distance (plus de 40 km) de **mai à août 2026**?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">How often did you or a member of your household make long-distance trips (more than 40 km) between **</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">May</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">August</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 2026**?</t>
+    </r>
   </si>
   <si>
     <r>
@@ -1918,11 +1967,60 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve"> de **septembre à décembre 2024**?</t>
+      <t xml:space="preserve"> de **mai à août 2026**?</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">How often did you make long-distance trips (more than 40 km) between **September and December 2024**?</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">How often did you make long-distance trips (more than 40 km) between **</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">May</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">August</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 2026**?</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">madeLongDistanceTripsConditional</t>
@@ -1937,7 +2035,7 @@
     <t xml:space="preserve">household.longDistanceTripsJanuaryApril</t>
   </si>
   <si>
-    <t xml:space="preserve">À quelle fréquence vous ou un des membres de votre ménage avez-vous effectué des déplacements longue distance (plus de 40 km) de **janvier à avril 2025**?</t>
+    <t xml:space="preserve">À quelle fréquence vous ou un des membres de votre ménage avez-vous effectué des déplacements longue distance (plus de 40 km) de **janvier à avril 2026**?</t>
   </si>
   <si>
     <r>
@@ -1988,7 +2086,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve"> 2025**?</t>
+      <t xml:space="preserve"> 2026**?</t>
     </r>
   </si>
   <si>
@@ -2020,7 +2118,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve"> de **janvier à avril 2025**?</t>
+      <t xml:space="preserve"> de **janvier à avril 2026**?</t>
     </r>
   </si>
   <si>
@@ -2072,69 +2170,20 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve"> 2025**?</t>
+      <t xml:space="preserve"> 2026**?</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">householdLongDistanceTripsMayAugust</t>
-  </si>
-  <si>
-    <t xml:space="preserve">household.longDistanceTripsMayAugust</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À quelle fréquence vous ou un des membres de votre ménage avez-vous effectué des déplacements longue distance (plus de 40 km) de **mai à août 2025**?</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Courier New"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">How often did you or a member of your household make long-distance trips (more than 40 km) between **</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">May</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Courier New"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> and </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">August</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Courier New"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 2025**?</t>
-    </r>
+    <t xml:space="preserve">householdLongDistanceTripsSeptemberDecember</t>
+  </si>
+  <si>
+    <t xml:space="preserve">household.longDistanceTripsSeptemberDecember</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À quelle fréquence vous ou un des membres de votre ménage avez-vous effectué des déplacements longue distance (plus de 40 km) de **septembre à décembre 2025**?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How often did you or a member of your household make long-distance trips (more than 40 km) between **September and December 2025**?</t>
   </si>
   <si>
     <r>
@@ -2165,60 +2214,11 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve"> de **mai à août 2025**?</t>
+      <t xml:space="preserve"> de **septembre à décembre 2025**?</t>
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Courier New"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">How often did you make long-distance trips (more than 40 km) between **</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">May</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Courier New"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> and </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">August</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Courier New"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 2025**?</t>
-    </r>
+    <t xml:space="preserve">How often did you make long-distance trips (more than 40 km) between **September and December 2025**?</t>
   </si>
   <si>
     <t xml:space="preserve">wouldLikeToParticipateToLongDistanceSurvey</t>
@@ -11470,6 +11470,33 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
+      <c r="XED113" s="0"/>
+      <c r="XEE113" s="0"/>
+      <c r="XEF113" s="0"/>
+      <c r="XEG113" s="0"/>
+      <c r="XEH113" s="0"/>
+      <c r="XEI113" s="0"/>
+      <c r="XEJ113" s="0"/>
+      <c r="XEK113" s="0"/>
+      <c r="XEL113" s="0"/>
+      <c r="XEM113" s="0"/>
+      <c r="XEN113" s="0"/>
+      <c r="XEO113" s="0"/>
+      <c r="XEP113" s="0"/>
+      <c r="XEQ113" s="0"/>
+      <c r="XER113" s="0"/>
+      <c r="XES113" s="0"/>
+      <c r="XET113" s="0"/>
+      <c r="XEU113" s="0"/>
+      <c r="XEV113" s="0"/>
+      <c r="XEW113" s="0"/>
+      <c r="XEX113" s="0"/>
+      <c r="XEY113" s="0"/>
+      <c r="XEZ113" s="0"/>
+      <c r="XFA113" s="0"/>
+      <c r="XFB113" s="0"/>
+      <c r="XFC113" s="0"/>
+      <c r="XFD113" s="0"/>
     </row>
     <row r="114" s="2" customFormat="true" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="40" t="s">
@@ -11644,7 +11671,7 @@
       <c r="P117" s="30"/>
       <c r="Q117" s="30"/>
       <c r="R117" s="30"/>
-      <c r="S117" s="28" t="n">
+      <c r="S117" s="28" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -12407,6 +12434,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <autoFilter ref="A1:W1"/>

</xml_diff>

<commit_message>
personDidTrips: ajout d'indications supplémentaires sur les déplacements
fixes #529

Ajout de la phrase "peu importe la distance parcourue ou le mode
de transport utilisé" dans le texte explication de la question, pour
clarifier le type de déplacements demandés.
</commit_message>
<xml_diff>
--- a/survey/references/OD_nationale_quebec_2025.xlsx
+++ b/survey/references/OD_nationale_quebec_2025.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -1033,20 +1033,96 @@
     <t xml:space="preserve">personDidTrips</t>
   </si>
   <si>
-    <t xml:space="preserve">Est-ce que {{nickname}} s'est déplac{{gender:é/ée/é(e)/é(e)}} le {{assignedDate}}?
-__Inclure tous les déplacements, qu'ils soient pour des motifs personnels (achats, sorties, loisirs, etc.), pour le travail, ou pour aller chercher ou reconduire quelqu'un.__</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Did {{nickname}} make any trips on {{assignedDate}}?
-__Include all trips, whether for personal reasons (shopping, outings, leisure, etc.), for work, or to pick up or drop someone off.__</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vous êtes-vous déplac{{gender:é/ée/é(e)/é(e)}} le {{assignedDate}}?
-__Inclure tous les déplacements, qu'ils soient pour des motifs personnels (achats, sorties, loisirs, etc.), pour le travail, ou pour aller chercher ou reconduire quelqu'un.__</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Did you make any trips on {{assignedDate}}?
-__Include all trips, whether for personal reasons (shopping, outings, leisure, etc.), for work, or to pick up or drop someone off.__</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Est-ce que {{nickname}} s'est déplac{{gender:é/ée/é(e)/é(e)}} le {{assignedDate}}?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">__Inclure tous les déplacements, peu importe la distance parcourue ou le mode de transport utilisé, qu'ils soient pour des motifs personnels (achats, sorties, loisirs, etc.), pour le travail, ou pour aller chercher ou reconduire quelqu'un.__</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Did {{nickname}} make any trips on {{assignedDate}}?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">__Include all trips, regardless of the distance travelled or mode of transportation used, whether for personal reasons (shopping, outings, leisure, etc.), for work, or to pick up or drop someone off.__</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Vous êtes-vous déplac{{gender:é/ée/é(e)/é(e)}} le {{assignedDate}}?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">__Inclure tous vos déplacements, peu importe la distance parcourue ou le mode de transport utilisé, qu'ils soient pour des motifs personnels (achats, sorties, loisirs, etc.), pour le travail, ou pour aller chercher ou reconduire quelqu'un.__</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Did you make any trips on {{assignedDate}}?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">__Include all trips, regardless of the distance travelled or mode of transportation used, whether for personal reasons (shopping, outings, leisure, etc.), for work, or to pick up or drop someone off.__</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">personDidTripsConfirm</t>
@@ -8691,7 +8767,7 @@
       <c r="V49" s="30"/>
       <c r="W49" s="30"/>
     </row>
-    <row r="50" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="140.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="10" t="s">
         <v>295</v>
       </c>

</xml_diff>